<commit_message>
done changes n reg
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Testdata.xlsx
+++ b/src/test/resources/testdata/Testdata.xlsx
@@ -7,15 +7,14 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="14180" windowHeight="5960"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Registration" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="12">
   <si>
     <t>FirstName</t>
   </si>
@@ -26,25 +25,31 @@
     <t>Email</t>
   </si>
   <si>
-    <t>Phone</t>
-  </si>
-  <si>
     <t>Password</t>
   </si>
   <si>
-    <t>ConfirmPassword</t>
-  </si>
-  <si>
-    <t>Ganesh</t>
-  </si>
-  <si>
-    <t>Kumar</t>
-  </si>
-  <si>
-    <t>ganesh@test.com</t>
-  </si>
-  <si>
-    <t>pass123</t>
+    <t>Telephone</t>
+  </si>
+  <si>
+    <t>PasswordConfirm</t>
+  </si>
+  <si>
+    <t>Newsletter</t>
+  </si>
+  <si>
+    <t>password123</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>ganesh</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>ganesh@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -413,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.90625" customWidth="1"/>
@@ -422,9 +427,10 @@
     <col min="4" max="4" width="25.81640625" customWidth="1"/>
     <col min="5" max="5" width="20.6328125" customWidth="1"/>
     <col min="6" max="6" width="16.90625" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -435,38 +441,116 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2">
-        <v>9999999999</v>
-      </c>
-      <c r="E2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="mailto:ganesh@test.com"/>
+    <hyperlink ref="C2" r:id="rId1"/>
+    <hyperlink ref="C3" r:id="rId2"/>
+    <hyperlink ref="C4" r:id="rId3"/>
+    <hyperlink ref="C5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>